<commit_message>
docs: record approximate 430-student DTS cohort
</commit_message>
<xml_diff>
--- a/A1_Current/UUse_A1_Market_Options_Evidence.xlsx
+++ b/A1_Current/UUse_A1_Market_Options_Evidence.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot model" sheetId="1" r:id="Rb97c22aa1222420b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R393b6c0089594614"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview review" sheetId="3" r:id="Rd7c24dbeceaf4f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot model" sheetId="1" r:id="Rbc8e8fd64f08437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rf581ff79b1434f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview review" sheetId="3" r:id="R3c3705b6ea12452f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
     <x:numFmt numFmtId="201" formatCode="#,##0&quot;+&quot;"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
@@ -23,6 +23,7 @@
     <x:numFmt numFmtId="204" formatCode="0%"/>
     <x:numFmt numFmtId="205" formatCode="0"/>
     <x:numFmt numFmtId="206" formatCode="0.00"/>
+    <x:numFmt numFmtId="207" formatCode="&quot;~&quot;#,##0"/>
   </x:numFmts>
   <x:fonts count="8">
     <x:font>
@@ -69,7 +70,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -91,6 +92,11 @@
         <x:fgColor rgb="FF28634E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -104,7 +110,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -181,6 +187,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -193,7 +208,7 @@
         <x:color rgb="FFA00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE0E0"/>
         </x:patternFill>
       </x:fill>
@@ -204,7 +219,7 @@
         <x:color rgb="FFA00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE0E0"/>
         </x:patternFill>
       </x:fill>
@@ -215,7 +230,7 @@
         <x:color rgb="FFA00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE0E0"/>
         </x:patternFill>
       </x:fill>
@@ -226,7 +241,7 @@
         <x:color rgb="FFA00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE0E0"/>
         </x:patternFill>
       </x:fill>
@@ -509,11 +524,11 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>DTS SAM, students</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:f>IF(COUNT(G18:G25)=B17,SUM(G18:G25),"Headcounts pending")</x:f>
-        <x:v>Headcounts pending</x:v>
+        <x:v>DTS cohort, students (approx.)</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="n">
+        <x:f>IF(COUNT(B35)=1,IF(B35&gt;=0,B35,"Invalid total"),IF(COUNT(G18:G25)=B17,SUM(G18:G25),"Cohort total pending"))</x:f>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2" t="str">
@@ -612,11 +627,11 @@
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2" t="str">
-        <x:v>Recruitment boundary</x:v>
+        <x:v>Invite count vs cohort</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:f>IF(COUNT(G18:G25)&lt;&gt;B17,"Reach unverified",IF(B7&gt;B6,"Invites exceed SAM","Within supplied SAM"))</x:f>
-        <x:v>Reach unverified</x:v>
+        <x:f>IF(ISNUMBER(B6),IF(B7&gt;B6,"Invites exceed cohort","Within reported cohort"),"Check cohort total")</x:f>
+        <x:v>Within reported cohort</x:v>
       </x:c>
       <x:c r="F11" s="2"/>
       <x:c r="G11" s="2"/>
@@ -631,8 +646,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
+      <x:c r="D12" s="2" t="str">
+        <x:v>Recruitment permission</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>To confirm</x:v>
+      </x:c>
       <x:c r="F12" s="2"/>
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
@@ -693,7 +712,7 @@
       <x:c r="E16" s="13"/>
       <x:c r="F16" s="13"/>
       <x:c r="G16" s="13" t="str">
-        <x:v>Eligible students</x:v>
+        <x:v>Per-class detail</x:v>
       </x:c>
       <x:c r="H16" s="13"/>
     </x:row>
@@ -730,7 +749,7 @@
       </x:c>
       <x:c r="G18" s="16"/>
       <x:c r="H18" s="13" t="str">
-        <x:v>Unique current headcounts, to be supplied.</x:v>
+        <x:v>Optional per-class breakdown. Do not invent counts.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -750,7 +769,7 @@
       </x:c>
       <x:c r="G19" s="16"/>
       <x:c r="H19" s="13" t="str">
-        <x:v>Do not replace unknown class sizes with zero.</x:v>
+        <x:v>Use the approximate aggregate in B35 until updated.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
@@ -770,7 +789,7 @@
       </x:c>
       <x:c r="G20" s="16"/>
       <x:c r="H20" s="13" t="str">
-        <x:v>Scope is eight classes, not 80 enrolled students.</x:v>
+        <x:v>80 invites are a planning target, not a class size.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
@@ -790,7 +809,7 @@
       </x:c>
       <x:c r="G21" s="16"/>
       <x:c r="H21" s="13" t="str">
-        <x:v>Invitations are separate planning assumptions.</x:v>
+        <x:v>Recruitment permission remains unconfirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
@@ -1010,10 +1029,16 @@
       <x:c r="H34" s="13"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
+      <x:c r="A35" s="2" t="str">
+        <x:v>Reported DTS cohort, students (approx.)</x:v>
+      </x:c>
+      <x:c r="B35" s="15" t="n">
+        <x:v>430</x:v>
+      </x:c>
       <x:c r="C35" s="2"/>
-      <x:c r="D35" s="2"/>
+      <x:c r="D35" s="2" t="str">
+        <x:v>Rita, 19 Oct 2026: about 430 students across eight DTS classes.</x:v>
+      </x:c>
       <x:c r="E35" s="2"/>
       <x:c r="F35" s="2"/>
       <x:c r="G35" s="2"/>
@@ -1038,7 +1063,7 @@
       <x:c r="B37" s="2"/>
       <x:c r="C37" s="2"/>
       <x:c r="D37" s="2" t="str">
-        <x:v>Rita, 15 October 2026: proposed pilot covers eight DTS classes. Class sizes, permission to recruit and unique reach have not been supplied. DTS is kept as provided, without an invented full programme name.</x:v>
+        <x:v>T1. Rita: eight DTS classes. The approximate cohort source is beside B35.</x:v>
       </x:c>
       <x:c r="E37" s="2"/>
       <x:c r="F37" s="2"/>

</xml_diff>

<commit_message>
docs: correct A1 market context to XEC campus population
</commit_message>
<xml_diff>
--- a/A1_Current/UUse_A1_Market_Options_Evidence.xlsx
+++ b/A1_Current/UUse_A1_Market_Options_Evidence.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot model" sheetId="1" r:id="Rbc8e8fd64f08437f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rf581ff79b1434f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview review" sheetId="3" r:id="R3c3705b6ea12452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot model" sheetId="1" r:id="Rb9d9756f38bb4931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R46a970866ac9486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview review" sheetId="3" r:id="Rbd27c5cacbee42bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,11 +504,11 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>Institutional universe, lower bound</x:v>
+        <x:v>XEC population context, reported</x:v>
       </x:c>
       <x:c r="B5" s="7" t="n">
         <x:f>B16</x:f>
-        <x:v>26000</x:v>
+        <x:v>4000</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
@@ -700,14 +700,14 @@
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>Institutional students, lower bound</x:v>
+        <x:v>XEC students, reported lower bound</x:v>
       </x:c>
       <x:c r="B16" s="15" t="n">
-        <x:v>26000</x:v>
+        <x:v>4000</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="13" t="str">
-        <x:v>S1. Institution-wide, not verified local demand.</x:v>
+        <x:v>S1. XEC only, May 2026 report. Population context, not measured demand.</x:v>
       </x:c>
       <x:c r="E16" s="13"/>
       <x:c r="F16" s="13"/>
@@ -1051,7 +1051,7 @@
       <x:c r="B36" s="2"/>
       <x:c r="C36" s="2"/>
       <x:c r="D36" s="2" t="str">
-        <x:v>XJTLU Overview &amp; Key Facts. https://www.xjtlu.edu.cn/en/overview . Accessed 15 October 2026. Institutional figure updated May 2026.</x:v>
+        <x:v>S1. XJTLU-hosted Xinhua Daily report, May 2026: 4,000+ XEC students. Not an October register.</x:v>
       </x:c>
       <x:c r="E36" s="2"/>
       <x:c r="F36" s="2"/>
@@ -1074,7 +1074,9 @@
       <x:c r="A38" s="2"/>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="2"/>
-      <x:c r="D38" s="2"/>
+      <x:c r="D38" s="2" t="str">
+        <x:v>https://www.xjtlu.edu.cn/zh/news/2026/05/xinhuaribao20zhounianxinwen</x:v>
+      </x:c>
       <x:c r="E38" s="2"/>
       <x:c r="F38" s="2"/>
       <x:c r="G38" s="2"/>

</xml_diff>